<commit_message>
Add Level-3 classification for financial customers
Map 金融客户 into tertiary categories from the taxonomy chart
(银行/券商/期货/基金/融资租赁/保险 sub-types) and export four columns.

Co-authored-by: Leo123456789011 <Leo123456789011@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/客户分类结果.xlsx
+++ b/客户分类结果.xlsx
@@ -11,7 +11,7 @@
     <sheet name="分类汇总" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'客户分类'!$A$1:$C$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'客户分类'!$A$1:$D$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,12 +480,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C164"/>
+  <dimension ref="A1:D164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +505,11 @@
           <t>二级分类</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>三级分类</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -521,6 +527,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -538,6 +549,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>政策性银行</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -555,6 +571,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -572,6 +593,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -589,6 +615,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -606,6 +637,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -623,6 +659,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -640,6 +681,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -657,6 +703,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>商业银行分行</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -674,6 +725,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>城市商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -691,6 +747,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -708,6 +769,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>城市商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -725,6 +791,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>城市商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -742,6 +813,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -759,6 +835,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -776,6 +857,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -793,6 +879,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>政策性银行</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -810,6 +901,11 @@
           <t>银行</t>
         </is>
       </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>商业银行</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -827,11 +923,16 @@
           <t>券商</t>
         </is>
       </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>东证融汇证券资产管理有限公司</t>
+          <t>五矿证券有限公司</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -842,13 +943,18 @@
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>五矿证券有限公司</t>
+          <t>中信建投证券股份有限公司</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -859,13 +965,18 @@
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>中信建投证券股份有限公司</t>
+          <t>中信证券股份有限公司</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -876,13 +987,18 @@
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>中信证券股份有限公司</t>
+          <t>中信证券股份有限公司辽宁分公司</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -893,13 +1009,18 @@
       <c r="C24" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>证券公司分公司</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>中信证券股份有限公司辽宁分公司</t>
+          <t>中信证券股份有限公司内蒙古分公司</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -910,13 +1031,18 @@
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>证券公司分公司</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>中信证券股份有限公司内蒙古分公司</t>
+          <t>中原证券股份有限公司</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -927,13 +1053,18 @@
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>中原证券股份有限公司</t>
+          <t>中天国富证券有限公司</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -944,13 +1075,18 @@
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>中天国富证券有限公司</t>
+          <t>中国银河证券股份有限公司</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -961,13 +1097,18 @@
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>中国银河证券股份有限公司</t>
+          <t>中泰证券股份有限公司</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -978,13 +1119,18 @@
       <c r="C29" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>中泰证券股份有限公司</t>
+          <t>中航证券有限公司</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -995,13 +1141,18 @@
       <c r="C30" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>中航证券有限公司</t>
+          <t>中金公司</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1012,13 +1163,18 @@
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>中金公司</t>
+          <t>中金财富证券有限公司</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1029,13 +1185,18 @@
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>中金财富证券有限公司</t>
+          <t>信达证券股份有限公司</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1046,13 +1207,18 @@
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>信达证券股份有限公司</t>
+          <t>华泰证券股份有限公司</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1063,13 +1229,18 @@
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>兴证证券资产管理有限公司</t>
+          <t>华安证券股份有限公司</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1080,13 +1251,18 @@
       <c r="C35" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>华泰证券股份有限公司</t>
+          <t>华融证券股份有限公司</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1097,13 +1273,18 @@
       <c r="C36" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>华安证券股份有限公司</t>
+          <t>国信证券股份有限公司</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1114,13 +1295,18 @@
       <c r="C37" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>华融证券股份有限公司</t>
+          <t>国泰君安证券股份有限公司</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1131,13 +1317,18 @@
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>国信证券股份有限公司</t>
+          <t>国金证券股份有限公司</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1148,13 +1339,18 @@
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>国泰君安证券股份有限公司</t>
+          <t>国元证券股份有限公司</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1165,13 +1361,18 @@
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>国金证券股份有限公司</t>
+          <t>国联证券股份有限公司</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1182,13 +1383,18 @@
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>国元证券股份有限公司</t>
+          <t>国海证券股份有限公司</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1199,13 +1405,18 @@
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>国联证券股份有限公司</t>
+          <t>国都证券股份有限公司</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1216,13 +1427,18 @@
       <c r="C43" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>国海证券股份有限公司</t>
+          <t>天风证券股份有限公司</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1233,13 +1449,18 @@
       <c r="C44" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>国都证券股份有限公司</t>
+          <t>安信证券股份有限公司</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1250,13 +1471,18 @@
       <c r="C45" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>天风证券股份有限公司</t>
+          <t>开源证券股份有限公司</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1267,13 +1493,18 @@
       <c r="C46" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>安信证券股份有限公司</t>
+          <t>招商证券股份有限公司</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1284,13 +1515,18 @@
       <c r="C47" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>开源证券股份有限公司</t>
+          <t>浙商证券股份有限公司</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1301,13 +1537,18 @@
       <c r="C48" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>招商证券股份有限公司</t>
+          <t>海通证券股份有限公司</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1318,13 +1559,18 @@
       <c r="C49" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>浙商证券股份有限公司</t>
+          <t>瑞银证券有限责任公司</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1335,13 +1581,18 @@
       <c r="C50" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>外资券商</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>海通证券股份有限公司</t>
+          <t>申万宏源证券有限公司</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1352,13 +1603,18 @@
       <c r="C51" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>瑞银证券有限责任公司</t>
+          <t>第一创业证券股份有限公司</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1369,13 +1625,18 @@
       <c r="C52" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>申万宏源证券有限公司</t>
+          <t>西部证券股份有限公司</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1386,13 +1647,18 @@
       <c r="C53" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>第一创业证券股份有限公司</t>
+          <t>银河证券</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1403,13 +1669,18 @@
       <c r="C54" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>证券公司</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>西部证券股份有限公司</t>
+          <t>摩根士丹利</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1420,13 +1691,18 @@
       <c r="C55" s="3" t="inlineStr">
         <is>
           <t>券商</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>外资券商</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>银河证券</t>
+          <t>中信期货有限公司</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -1436,14 +1712,19 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>券商</t>
+          <t>期货</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>期货公司</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>摩根士丹利</t>
+          <t>冠通期货股份有限公司</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1453,14 +1734,19 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>券商</t>
+          <t>期货</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>期货公司</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>中信期货有限公司</t>
+          <t>华泰期货有限公司</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1471,13 +1757,18 @@
       <c r="C58" s="3" t="inlineStr">
         <is>
           <t>期货</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>期货公司</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>冠通期货股份有限公司</t>
+          <t>南华期货股份有限公司</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1488,13 +1779,18 @@
       <c r="C59" s="3" t="inlineStr">
         <is>
           <t>期货</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>期货公司</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>华泰期货有限公司</t>
+          <t>中金基金管理有限公司</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -1504,14 +1800,19 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>期货</t>
+          <t>基金</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>南华期货股份有限公司</t>
+          <t>华安基金管理有限公司</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1521,14 +1822,19 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>期货</t>
+          <t>基金</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>中金基金管理有限公司</t>
+          <t>华夏基金管理有限公司</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1539,13 +1845,18 @@
       <c r="C62" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>华安基金管理有限公司</t>
+          <t>博时基金管理有限公司</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1556,13 +1867,18 @@
       <c r="C63" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>华夏基金管理有限公司</t>
+          <t>工银瑞信基金管理有限公司</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1573,13 +1889,18 @@
       <c r="C64" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>博时基金管理有限公司</t>
+          <t>建信基金管理有限公司</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1590,13 +1911,18 @@
       <c r="C65" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>工银瑞信基金管理有限公司</t>
+          <t>易方达基金管理有限公司</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -1607,13 +1933,18 @@
       <c r="C66" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>公募基金</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>建信基金管理有限公司</t>
+          <t>东证融汇证券资产管理有限公司</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -1624,13 +1955,18 @@
       <c r="C67" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>券商私募（另类投资）</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>易方达基金管理有限公司</t>
+          <t>兴证证券资产管理有限公司</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -1641,6 +1977,11 @@
       <c r="C68" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>券商私募（另类投资）</t>
         </is>
       </c>
     </row>
@@ -1660,6 +2001,11 @@
           <t>基金</t>
         </is>
       </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1677,6 +2023,11 @@
           <t>基金</t>
         </is>
       </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1694,6 +2045,11 @@
           <t>基金</t>
         </is>
       </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1711,11 +2067,16 @@
           <t>基金</t>
         </is>
       </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>中信资本控股有限公司</t>
+          <t>中信资本股权投资管理有限公司</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -1726,13 +2087,18 @@
       <c r="C73" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>中信资本股权投资管理有限公司</t>
+          <t>中投保信投资管理有限公司</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -1743,13 +2109,18 @@
       <c r="C74" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>中国银河投资管理有限公司</t>
+          <t>凯雷（北京）投资管理有限公司</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -1760,13 +2131,18 @@
       <c r="C75" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>中投保信投资管理有限公司</t>
+          <t>上海微策金融信息服务有限公司</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -1777,13 +2153,18 @@
       <c r="C76" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>私募基金</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>中融国际信托有限公司</t>
+          <t>中信资本控股有限公司</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -1794,13 +2175,18 @@
       <c r="C77" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>私募投资集团</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>凯雷（北京）投资管理有限公司</t>
+          <t>中国银河投资管理有限公司</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -1811,13 +2197,18 @@
       <c r="C78" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>私募投资集团</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>宜信</t>
+          <t>中融国际信托有限公司</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -1828,13 +2219,18 @@
       <c r="C79" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>私募投资集团</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>上海微策金融信息服务有限公司</t>
+          <t>宜信</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -1845,6 +2241,11 @@
       <c r="C80" s="3" t="inlineStr">
         <is>
           <t>基金</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>私募投资集团</t>
         </is>
       </c>
     </row>
@@ -1864,6 +2265,11 @@
           <t>融资租赁</t>
         </is>
       </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>融资租赁</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1881,6 +2287,11 @@
           <t>融资租赁</t>
         </is>
       </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>融资租赁</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1898,6 +2309,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1915,6 +2331,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -1932,6 +2353,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1949,6 +2375,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -1966,6 +2397,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1983,6 +2419,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2000,6 +2441,11 @@
           <t>保险</t>
         </is>
       </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>保险集团</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2017,6 +2463,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2034,6 +2481,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2051,6 +2499,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2068,6 +2517,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2085,6 +2535,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2102,6 +2553,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2119,6 +2571,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2136,6 +2589,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2153,6 +2607,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2170,6 +2625,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2187,6 +2643,7 @@
           <t>采矿业</t>
         </is>
       </c>
+      <c r="D100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2204,6 +2661,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2221,6 +2679,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2238,6 +2697,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2255,6 +2715,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -2272,6 +2733,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -2289,6 +2751,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -2306,6 +2769,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -2323,6 +2787,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -2340,6 +2805,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -2357,6 +2823,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -2374,6 +2841,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -2391,6 +2859,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -2408,6 +2877,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -2425,6 +2895,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2442,6 +2913,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -2459,6 +2931,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -2476,6 +2949,7 @@
           <t>制造业</t>
         </is>
       </c>
+      <c r="D117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -2493,6 +2967,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D118" s="4" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -2510,6 +2985,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -2527,6 +3003,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -2544,6 +3021,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -2561,6 +3039,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -2578,6 +3057,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -2595,6 +3075,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -2612,6 +3093,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -2629,6 +3111,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -2646,6 +3129,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -2663,6 +3147,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -2680,6 +3165,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -2697,6 +3183,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D130" s="4" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -2714,6 +3201,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -2731,6 +3219,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D132" s="4" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -2748,6 +3237,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -2765,6 +3255,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2782,6 +3273,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -2799,6 +3291,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -2816,6 +3309,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -2833,6 +3327,7 @@
           <t>服务业</t>
         </is>
       </c>
+      <c r="D138" s="4" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -2850,6 +3345,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -2867,6 +3363,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -2884,6 +3381,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -2901,6 +3399,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D142" s="4" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -2918,6 +3417,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -2935,6 +3435,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D144" s="4" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -2952,6 +3453,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -2969,6 +3471,7 @@
           <t>建筑业</t>
         </is>
       </c>
+      <c r="D146" s="4" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -2986,6 +3489,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D147" s="4" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -3003,6 +3507,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D148" s="4" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -3020,6 +3525,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -3037,6 +3543,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D150" s="4" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -3054,6 +3561,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D151" s="4" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -3071,6 +3579,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D152" s="4" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -3088,6 +3597,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -3105,6 +3615,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D154" s="4" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -3122,6 +3633,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -3139,6 +3651,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D156" s="4" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -3156,6 +3669,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D157" s="4" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -3173,6 +3687,7 @@
           <t>贸易业</t>
         </is>
       </c>
+      <c r="D158" s="4" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -3190,6 +3705,7 @@
           <t>其他</t>
         </is>
       </c>
+      <c r="D159" s="4" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -3207,6 +3723,7 @@
           <t>个人客户</t>
         </is>
       </c>
+      <c r="D160" s="5" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -3224,6 +3741,7 @@
           <t>个人客户</t>
         </is>
       </c>
+      <c r="D161" s="5" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -3241,6 +3759,7 @@
           <t>个人客户</t>
         </is>
       </c>
+      <c r="D162" s="5" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -3258,6 +3777,7 @@
           <t>其他</t>
         </is>
       </c>
+      <c r="D163" s="6" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -3275,9 +3795,10 @@
           <t>其他</t>
         </is>
       </c>
+      <c r="D164" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C164"/>
+  <autoFilter ref="A1:D164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3292,7 +3813,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -3361,12 +3882,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>一级分类</t>
+          <t>二级分类</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>二级分类</t>
+          <t>三级分类</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -3378,211 +3899,211 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>个人客户</t>
+          <t>保险</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>个人客户</t>
+          <t>保险集团</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>券商</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>外资券商</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>券商</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>制造业</t>
+          <t>证券公司</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>券商</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>建筑业</t>
+          <t>证券公司分公司</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>服务业</t>
+          <t>公募基金</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>贸易业</t>
+          <t>券商私募（另类投资）</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>产业客户</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>采矿业</t>
+          <t>私募基金</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>基金</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>私募投资集团</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>期货</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>保险</t>
+          <t>期货公司</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>融资租赁</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>券商</t>
+          <t>融资租赁</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>基金</t>
+          <t>商业银行</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>期货</t>
+          <t>商业银行分行</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>融资租赁</t>
+          <t>城市商业银行</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>金融客户</t>
+          <t>银行</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>银行</t>
+          <t>政策性银行</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>